<commit_message>
Regenerate project artifacts with linkml 1.11
The JSON schema now carries format: uri on dataset_url and
bibliographicCitation, which are declared range: uri.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/excel/brc_schema.xlsx
+++ b/project/excel/brc_schema.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DatasetCollection" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dataset" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Individual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="OntologyAnnotation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Contributor" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Funding" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="BRCOrganization" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Organism" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Plasmid" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="RelatedItem" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="MediaSet" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="MediaFile" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DatasetCollection" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Individual" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OntologyAnnotation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contributor" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BRCOrganization" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organism" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plasmid" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RelatedItem" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediaSet" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediaFile" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>